<commit_message>
updating for 11 sept
</commit_message>
<xml_diff>
--- a/1234567.xlsx
+++ b/1234567.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satya\Desktop\datasheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D608A5E8-6A67-4373-9B1A-A4E12B5B189C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1293944-3D64-4B6C-B68E-B7D0BABF8E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="66">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2317,24 +2317,44 @@
       <c r="N36" s="17"/>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
+      <c r="A37" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B37" s="14">
+        <v>100</v>
+      </c>
+      <c r="C37" s="14">
+        <v>60</v>
+      </c>
+      <c r="D37" s="14">
+        <v>0</v>
+      </c>
+      <c r="E37" s="14">
+        <v>15</v>
+      </c>
+      <c r="F37" s="14">
+        <v>2</v>
+      </c>
+      <c r="G37" s="14">
+        <v>2</v>
+      </c>
+      <c r="H37" s="14">
+        <v>60</v>
+      </c>
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
+        <v>237</v>
+      </c>
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
+        <v>1203</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>65</v>
+      </c>
       <c r="M37" s="16"/>
       <c r="N37" s="17"/>
     </row>

</xml_diff>